<commit_message>
Sync card_data.xlsx renames and Lex Purgatoria into game data.
Rename nine units that kept matching stats/effects under new names, update vaults/packs/tests/refs, add Lex Purgatoria, and sync remaining xlsx stats.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/context/card_data.xlsx
+++ b/context/card_data.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="2100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="2102">
   <si>
     <t>Table 1</t>
   </si>
@@ -391,7 +391,7 @@
     <t>Ice Mage</t>
   </si>
   <si>
-    <t>Asteroid Trooper</t>
+    <t>Star Hunter</t>
   </si>
   <si>
     <t>Slim Gray Tank</t>
@@ -877,7 +877,7 @@
     <t>Skeleton Sickleman</t>
   </si>
   <si>
-    <t>Human Dog</t>
+    <t>Kappa</t>
   </si>
   <si>
     <t>+10 ATK if there is Anima or Nature card on your side</t>
@@ -1207,7 +1207,7 @@
     <t>Mad Raccoon</t>
   </si>
   <si>
-    <t>Armored Monkey</t>
+    <t>Armored Cat</t>
   </si>
   <si>
     <t>+10 ATK if there is another exposed Nature card</t>
@@ -1678,10 +1678,10 @@
     <t>Zetamas the Great Summoner</t>
   </si>
   <si>
-    <t>At the end of your turn: create a token copy of Leviathan on an empty cell on your side</t>
-  </si>
-  <si>
-    <t>Ethereal Shielder</t>
+    <t>When this card is exposed, you can choose to summon 1 Mad Wyvern token on any of your cell.</t>
+  </si>
+  <si>
+    <t>Ethereal Soldiers</t>
   </si>
   <si>
     <t>Once per turn, this card cannot be destroyed vs Non-Arcane</t>
@@ -1762,7 +1762,7 @@
     <t>Sweet Lure Pod</t>
   </si>
   <si>
-    <t>This turn, foe can only target this card for an attack.</t>
+    <t>Foe can only target this exposed card for an attack.</t>
   </si>
   <si>
     <t>Radiaghoul</t>
@@ -1825,16 +1825,16 @@
     <t>S-02 the Hatcher</t>
   </si>
   <si>
-    <t>Once at foe’s turn end, create a token on an empty cell with 0 ATK&amp;DEF and no ability.</t>
-  </si>
-  <si>
-    <t>Rotten Shrieker</t>
+    <t>Once at foe’s turn end, create a token on an empty cell with 0 ATK&amp;DEF, no cost, and no ability</t>
+  </si>
+  <si>
+    <t>Rotten Spider</t>
   </si>
   <si>
     <t>Without Mutagen Flag : -10 ATK permanently at the end of your turn.</t>
   </si>
   <si>
-    <t>Toxin Folk</t>
+    <t>Toxin Eater</t>
   </si>
   <si>
     <t>While this card is exposed, foe that perform attack get -5 ATK until the end of foe’s turn.</t>
@@ -1891,10 +1891,10 @@
     <t>After successfully attacking, flip a coin, if head, gain 50 Crystal</t>
   </si>
   <si>
-    <t>Epsilon The Wither</t>
-  </si>
-  <si>
-    <t>At Reckoning, +40 ATK&amp;DEF until this turn ends, but all ally units lose 10 ATK&amp;DEF until this turn ends</t>
+    <t>Epsilon The Withered</t>
+  </si>
+  <si>
+    <t>At Reckoning, +40 ATK&amp;DEF until this turn ends, but all ally units lose 40 ATK&amp;DEF until foe’s turn ends</t>
   </si>
   <si>
     <t>Plaguespreader</t>
@@ -1903,7 +1903,7 @@
     <t>With Mutagen Flag : At the end of your turn, put 1 Mutagen Flag on one of your exposed card.</t>
   </si>
   <si>
-    <t>Black Worms</t>
+    <t>Slug-11</t>
   </si>
   <si>
     <t>At your turn’s end, foe loses 300 Crystals for each Mutagen flag on the field</t>
@@ -2026,10 +2026,10 @@
     <t>Exposed: Reveal 1 of your own cells</t>
   </si>
   <si>
-    <t>Aembar the Intel Dealer</t>
-  </si>
-  <si>
-    <t>Any player use Tech card, they reveal 1 cell on their field. Usable face-down.</t>
+    <t>Aembar the Intel Broker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any player lose or pay crystals, they reveal 1 cell on their field. Usable face-down. </t>
   </si>
   <si>
     <t>Tholin Lobster</t>
@@ -6762,6 +6762,12 @@
   </si>
   <si>
     <t>Relocate two of foe’s face-up units</t>
+  </si>
+  <si>
+    <t>Lex Purgatoria</t>
+  </si>
+  <si>
+    <t>Until the end of foe’s turn, destroy any Arcane unit in Reckoning with Anima units.</t>
   </si>
   <si>
     <t>Expected</t>
@@ -20501,7 +20507,7 @@
         <v>33</v>
       </c>
       <c r="C296" s="18">
-        <v>1200</v>
+        <v>820</v>
       </c>
       <c r="D296" s="18">
         <v>55</v>
@@ -20519,7 +20525,9 @@
         <v>549</v>
       </c>
       <c r="I296" s="12"/>
-      <c r="J296" s="12"/>
+      <c r="J296" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K296" s="18">
         <f>(D296*6)+(E296*4)</f>
         <v>670</v>
@@ -20556,7 +20564,9 @@
         <v>551</v>
       </c>
       <c r="I297" s="12"/>
-      <c r="J297" s="12"/>
+      <c r="J297" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K297" s="18">
         <f>(D297*6)+(E297*4)</f>
         <v>540</v>
@@ -20567,7 +20577,7 @@
       <c r="O297" s="12"/>
       <c r="P297" s="12"/>
     </row>
-    <row r="298" ht="44.05" customHeight="1">
+    <row r="298" ht="56.4" customHeight="1">
       <c r="A298" t="s" s="10">
         <v>552</v>
       </c>
@@ -20575,13 +20585,13 @@
         <v>33</v>
       </c>
       <c r="C298" s="18">
-        <v>1000</v>
+        <v>600</v>
       </c>
       <c r="D298" s="18">
         <v>0</v>
       </c>
       <c r="E298" s="18">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="F298" t="s" s="19">
         <v>7</v>
@@ -20593,10 +20603,12 @@
         <v>553</v>
       </c>
       <c r="I298" s="12"/>
-      <c r="J298" s="12"/>
+      <c r="J298" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K298" s="18">
         <f>(D298*6)+(E298*4)</f>
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="L298" s="12"/>
       <c r="M298" s="12"/>
@@ -20630,7 +20642,9 @@
         <v>555</v>
       </c>
       <c r="I299" s="12"/>
-      <c r="J299" s="12"/>
+      <c r="J299" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K299" s="18">
         <f>(D299*6)+(E299*4)</f>
         <v>470</v>
@@ -20667,7 +20681,9 @@
         <v>557</v>
       </c>
       <c r="I300" s="12"/>
-      <c r="J300" s="12"/>
+      <c r="J300" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K300" s="18">
         <f>(D300*6)+(E300*4)</f>
         <v>1190</v>
@@ -20704,7 +20720,9 @@
         <v>559</v>
       </c>
       <c r="I301" s="12"/>
-      <c r="J301" s="12"/>
+      <c r="J301" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K301" s="18">
         <f>(D301*6)+(E301*4)</f>
         <v>1580</v>
@@ -20741,7 +20759,9 @@
         <v>561</v>
       </c>
       <c r="I302" s="12"/>
-      <c r="J302" s="12"/>
+      <c r="J302" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K302" s="18">
         <f>(D302*6)+(E302*4)</f>
         <v>870</v>
@@ -20763,10 +20783,10 @@
         <v>2000</v>
       </c>
       <c r="D303" s="18">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="E303" s="18">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="F303" t="s" s="19">
         <v>7</v>
@@ -20778,10 +20798,12 @@
         <v>563</v>
       </c>
       <c r="I303" s="12"/>
-      <c r="J303" s="12"/>
+      <c r="J303" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K303" s="18">
         <f>(D303*6)+(E303*4)</f>
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="L303" s="12"/>
       <c r="M303" s="12"/>
@@ -20901,7 +20923,9 @@
         <v>39</v>
       </c>
       <c r="I306" s="12"/>
-      <c r="J306" s="12"/>
+      <c r="J306" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K306" s="18">
         <f>(D306*6)+(E306*4)</f>
         <v>150</v>
@@ -20981,7 +21005,9 @@
         <v>39</v>
       </c>
       <c r="I308" s="12"/>
-      <c r="J308" s="12"/>
+      <c r="J308" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K308" s="18">
         <f>(D308*6)+(E308*4)</f>
         <v>220</v>
@@ -21061,7 +21087,9 @@
         <v>575</v>
       </c>
       <c r="I310" s="12"/>
-      <c r="J310" s="12"/>
+      <c r="J310" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K310" s="18">
         <f>(D310*6)+(E310*4)</f>
         <v>100</v>
@@ -21139,7 +21167,9 @@
         <v>579</v>
       </c>
       <c r="I312" s="12"/>
-      <c r="J312" s="12"/>
+      <c r="J312" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K312" s="18">
         <f>(D312*6)+(E312*4)</f>
         <v>140</v>
@@ -21176,7 +21206,9 @@
         <v>581</v>
       </c>
       <c r="I313" s="12"/>
-      <c r="J313" s="12"/>
+      <c r="J313" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K313" s="18">
         <f>(D313*6)+(E313*4)</f>
         <v>120</v>
@@ -21342,7 +21374,9 @@
         <v>589</v>
       </c>
       <c r="I317" s="12"/>
-      <c r="J317" s="12"/>
+      <c r="J317" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K317" s="18">
         <f>(D317*6)+(E317*4)</f>
         <v>0</v>
@@ -21422,7 +21456,9 @@
         <v>39</v>
       </c>
       <c r="I319" s="12"/>
-      <c r="J319" s="12"/>
+      <c r="J319" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K319" s="18">
         <f>(D319*6)+(E319*4)</f>
         <v>170</v>
@@ -21459,7 +21495,9 @@
         <v>594</v>
       </c>
       <c r="I320" s="12"/>
-      <c r="J320" s="12"/>
+      <c r="J320" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K320" s="18">
         <f>(D320*6)+(E320*4)</f>
         <v>80</v>
@@ -21496,7 +21534,9 @@
         <v>596</v>
       </c>
       <c r="I321" s="12"/>
-      <c r="J321" s="12"/>
+      <c r="J321" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K321" s="18">
         <f>(D321*6)+(E321*4)</f>
         <v>230</v>
@@ -21533,7 +21573,9 @@
         <v>39</v>
       </c>
       <c r="I322" s="12"/>
-      <c r="J322" s="12"/>
+      <c r="J322" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K322" s="18">
         <f>(D322*6)+(E322*4)</f>
         <v>280</v>
@@ -21656,7 +21698,9 @@
         <v>602</v>
       </c>
       <c r="I325" s="12"/>
-      <c r="J325" s="12"/>
+      <c r="J325" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K325" s="18">
         <f>(D325*6)+(E325*4)</f>
         <v>170</v>
@@ -21736,7 +21780,9 @@
         <v>606</v>
       </c>
       <c r="I327" s="12"/>
-      <c r="J327" s="12"/>
+      <c r="J327" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K327" s="18">
         <f>(D327*6)+(E327*4)</f>
         <v>250</v>
@@ -21773,7 +21819,9 @@
         <v>39</v>
       </c>
       <c r="I328" s="12"/>
-      <c r="J328" s="12"/>
+      <c r="J328" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K328" s="18">
         <f>(D328*6)+(E328*4)</f>
         <v>120</v>
@@ -21896,7 +21944,9 @@
         <v>39</v>
       </c>
       <c r="I331" s="12"/>
-      <c r="J331" s="12"/>
+      <c r="J331" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K331" s="18">
         <f>(D331*6)+(E331*4)</f>
         <v>550</v>
@@ -21937,7 +21987,9 @@
         <v>614</v>
       </c>
       <c r="I332" s="12"/>
-      <c r="J332" s="12"/>
+      <c r="J332" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K332" s="18">
         <f>(D332*6)+(E332*4)</f>
         <v>520</v>
@@ -21974,7 +22026,9 @@
         <v>616</v>
       </c>
       <c r="I333" s="12"/>
-      <c r="J333" s="12"/>
+      <c r="J333" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K333" s="18">
         <f>(D333*6)+(E333*4)</f>
         <v>660</v>
@@ -22011,7 +22065,9 @@
         <v>39</v>
       </c>
       <c r="I334" s="12"/>
-      <c r="J334" s="12"/>
+      <c r="J334" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K334" s="18">
         <f>(D334*6)+(E334*4)</f>
         <v>600</v>
@@ -22048,7 +22104,9 @@
         <v>619</v>
       </c>
       <c r="I335" s="12"/>
-      <c r="J335" s="12"/>
+      <c r="J335" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K335" s="18">
         <f>(D335*6)+(E335*4)</f>
         <v>360</v>
@@ -22085,7 +22143,9 @@
         <v>621</v>
       </c>
       <c r="I336" s="12"/>
-      <c r="J336" s="12"/>
+      <c r="J336" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K336" s="18">
         <f>(D336*6)+(E336*4)</f>
         <v>400</v>
@@ -22122,7 +22182,9 @@
         <v>623</v>
       </c>
       <c r="I337" s="12"/>
-      <c r="J337" s="12"/>
+      <c r="J337" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K337" s="18">
         <f>(D337*6)+(E337*4)</f>
         <v>690</v>
@@ -22159,7 +22221,9 @@
         <v>625</v>
       </c>
       <c r="I338" s="12"/>
-      <c r="J338" s="12"/>
+      <c r="J338" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K338" s="18">
         <f>(D338*6)+(E338*4)</f>
         <v>680</v>
@@ -22196,7 +22260,9 @@
         <v>627</v>
       </c>
       <c r="I339" s="12"/>
-      <c r="J339" s="12"/>
+      <c r="J339" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K339" s="18">
         <f>(D339*6)+(E339*4)</f>
         <v>590</v>
@@ -22276,7 +22342,9 @@
         <v>631</v>
       </c>
       <c r="I341" s="12"/>
-      <c r="J341" s="12"/>
+      <c r="J341" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K341" s="18">
         <f>(D341*6)+(E341*4)</f>
         <v>520</v>
@@ -22313,7 +22381,9 @@
         <v>633</v>
       </c>
       <c r="I342" s="12"/>
-      <c r="J342" s="12"/>
+      <c r="J342" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K342" s="18">
         <f>(D342*6)+(E342*4)</f>
         <v>540</v>
@@ -22350,7 +22420,9 @@
         <v>635</v>
       </c>
       <c r="I343" s="12"/>
-      <c r="J343" s="12"/>
+      <c r="J343" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K343" s="18">
         <f>(D343*6)+(E343*4)</f>
         <v>990</v>
@@ -22387,7 +22459,9 @@
         <v>637</v>
       </c>
       <c r="I344" s="12"/>
-      <c r="J344" s="12"/>
+      <c r="J344" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K344" s="18">
         <f>(D344*6)+(E344*4)</f>
         <v>800</v>
@@ -22424,7 +22498,9 @@
         <v>639</v>
       </c>
       <c r="I345" s="12"/>
-      <c r="J345" s="12"/>
+      <c r="J345" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K345" s="18">
         <f>(D345*6)+(E345*4)</f>
         <v>750</v>
@@ -22461,7 +22537,9 @@
         <v>641</v>
       </c>
       <c r="I346" s="12"/>
-      <c r="J346" s="12"/>
+      <c r="J346" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K346" s="18">
         <f>(D346*6)+(E346*4)</f>
         <v>1200</v>
@@ -22486,7 +22564,7 @@
         <v>40</v>
       </c>
       <c r="E347" s="18">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="F347" t="s" s="19">
         <v>11</v>
@@ -22498,10 +22576,12 @@
         <v>643</v>
       </c>
       <c r="I347" s="12"/>
-      <c r="J347" s="12"/>
+      <c r="J347" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K347" s="18">
         <f>(D347*6)+(E347*4)</f>
-        <v>540</v>
+        <v>440</v>
       </c>
       <c r="L347" s="12"/>
       <c r="M347" s="12"/>
@@ -22535,7 +22615,9 @@
         <v>39</v>
       </c>
       <c r="I348" s="12"/>
-      <c r="J348" s="12"/>
+      <c r="J348" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K348" s="18">
         <f>(D348*6)+(E348*4)</f>
         <v>1150</v>
@@ -22744,7 +22826,9 @@
         <v>654</v>
       </c>
       <c r="I353" s="12"/>
-      <c r="J353" s="12"/>
+      <c r="J353" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K353" s="18">
         <f>(D353*6)+(E353*4)</f>
         <v>120</v>
@@ -22781,7 +22865,9 @@
         <v>656</v>
       </c>
       <c r="I354" s="12"/>
-      <c r="J354" s="12"/>
+      <c r="J354" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K354" s="18">
         <f>(D354*6)+(E354*4)</f>
         <v>100</v>
@@ -22818,7 +22904,9 @@
         <v>39</v>
       </c>
       <c r="I355" s="12"/>
-      <c r="J355" s="12"/>
+      <c r="J355" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K355" s="18">
         <f>(D355*6)+(E355*4)</f>
         <v>190</v>
@@ -22855,7 +22943,9 @@
         <v>39</v>
       </c>
       <c r="I356" s="12"/>
-      <c r="J356" s="12"/>
+      <c r="J356" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K356" s="18">
         <f>(D356*6)+(E356*4)</f>
         <v>230</v>
@@ -22892,7 +22982,9 @@
         <v>660</v>
       </c>
       <c r="I357" s="12"/>
-      <c r="J357" s="12"/>
+      <c r="J357" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K357" s="18">
         <f>(D357*6)+(E357*4)</f>
         <v>190</v>
@@ -22929,7 +23021,9 @@
         <v>662</v>
       </c>
       <c r="I358" s="12"/>
-      <c r="J358" s="12"/>
+      <c r="J358" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K358" s="18">
         <f>(D358*6)+(E358*4)</f>
         <v>100</v>
@@ -22966,7 +23060,9 @@
         <v>664</v>
       </c>
       <c r="I359" s="12"/>
-      <c r="J359" s="12"/>
+      <c r="J359" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K359" s="18">
         <f>(D359*6)+(E359*4)</f>
         <v>140</v>
@@ -23003,7 +23099,9 @@
         <v>666</v>
       </c>
       <c r="I360" s="12"/>
-      <c r="J360" s="12"/>
+      <c r="J360" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K360" s="18">
         <f>(D360*6)+(E360*4)</f>
         <v>180</v>
@@ -23040,7 +23138,9 @@
         <v>668</v>
       </c>
       <c r="I361" s="12"/>
-      <c r="J361" s="12"/>
+      <c r="J361" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K361" s="18">
         <f>(D361*6)+(E361*4)</f>
         <v>220</v>
@@ -23051,7 +23151,7 @@
       <c r="O361" s="12"/>
       <c r="P361" s="12"/>
     </row>
-    <row r="362" ht="32.05" customHeight="1">
+    <row r="362" ht="38.7" customHeight="1">
       <c r="A362" t="s" s="10">
         <v>669</v>
       </c>
@@ -23059,7 +23159,7 @@
         <v>33</v>
       </c>
       <c r="C362" s="18">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="D362" s="18">
         <v>10</v>
@@ -23077,7 +23177,9 @@
         <v>670</v>
       </c>
       <c r="I362" s="12"/>
-      <c r="J362" s="12"/>
+      <c r="J362" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K362" s="18">
         <f>(D362*6)+(E362*4)</f>
         <v>100</v>
@@ -23114,7 +23216,9 @@
         <v>672</v>
       </c>
       <c r="I363" s="12"/>
-      <c r="J363" s="12"/>
+      <c r="J363" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K363" s="18">
         <f>(D363*6)+(E363*4)</f>
         <v>150</v>
@@ -23151,7 +23255,9 @@
         <v>674</v>
       </c>
       <c r="I364" s="12"/>
-      <c r="J364" s="12"/>
+      <c r="J364" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K364" s="18">
         <f>(D364*6)+(E364*4)</f>
         <v>200</v>
@@ -23317,7 +23423,9 @@
         <v>682</v>
       </c>
       <c r="I368" s="12"/>
-      <c r="J368" s="12"/>
+      <c r="J368" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K368" s="18">
         <f>(D368*6)+(E368*4)</f>
         <v>120</v>
@@ -50328,14 +50436,22 @@
       <c r="P132" s="12"/>
     </row>
     <row r="133" ht="20.05" customHeight="1">
-      <c r="A133" s="13"/>
-      <c r="B133" s="14"/>
-      <c r="C133" s="12"/>
+      <c r="A133" t="s" s="10">
+        <v>2067</v>
+      </c>
+      <c r="B133" t="s" s="11">
+        <v>1806</v>
+      </c>
+      <c r="C133" s="18">
+        <v>800</v>
+      </c>
       <c r="D133" s="12"/>
       <c r="E133" s="12"/>
       <c r="F133" s="12"/>
       <c r="G133" s="12"/>
-      <c r="H133" s="12"/>
+      <c r="H133" t="s" s="19">
+        <v>2068</v>
+      </c>
       <c r="I133" s="12"/>
       <c r="J133" s="12"/>
       <c r="K133" s="12"/>
@@ -57800,21 +57916,21 @@
         <v>22</v>
       </c>
       <c r="B2" t="s" s="37">
-        <v>2067</v>
+        <v>2069</v>
       </c>
       <c r="C2" t="s" s="37">
-        <v>2068</v>
+        <v>2070</v>
       </c>
       <c r="D2" t="s" s="37">
-        <v>2069</v>
+        <v>2071</v>
       </c>
       <c r="E2" t="s" s="37">
-        <v>2070</v>
+        <v>2072</v>
       </c>
     </row>
     <row r="3" ht="16.55" customHeight="1">
       <c r="A3" t="s" s="38">
-        <v>2071</v>
+        <v>2073</v>
       </c>
       <c r="B3" s="39">
         <v>52</v>
@@ -57823,16 +57939,16 @@
         <v>0.347</v>
       </c>
       <c r="D3" t="s" s="41">
-        <v>2072</v>
+        <v>2074</v>
       </c>
       <c r="E3" s="42">
         <f>_xlfn.COUNTIFS('Unit'!$J$3:$J$599,"Yes",'Unit'!$G$3:$G$599,1)+_xlfn.COUNTIFS('Trap'!$J$3:$J$544,"Yes",'Trap'!$G$3:$G$544,1)+_xlfn.COUNTIFS('Tech'!$J$3:$J$545,"Yes",'Tech'!$G$3:$G$545,1)</f>
-        <v>112</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" ht="16.35" customHeight="1">
       <c r="A4" t="s" s="43">
-        <v>2073</v>
+        <v>2075</v>
       </c>
       <c r="B4" s="44">
         <v>48</v>
@@ -57841,16 +57957,16 @@
         <v>0.337</v>
       </c>
       <c r="D4" t="s" s="46">
-        <v>2074</v>
+        <v>2076</v>
       </c>
       <c r="E4" s="47">
         <f>_xlfn.COUNTIFS('Unit'!$J$3:$J$599,"Yes",'Unit'!$G$3:$G$599,2)+_xlfn.COUNTIFS('Trap'!$J$3:$J$544,"Yes",'Trap'!$G$3:$G$544,2)+_xlfn.COUNTIFS('Tech'!$J$3:$J$545,"Yes",'Tech'!$G$3:$G$545,2)</f>
-        <v>104</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" ht="16.35" customHeight="1">
       <c r="A5" t="s" s="43">
-        <v>2075</v>
+        <v>2077</v>
       </c>
       <c r="B5" s="44">
         <v>27</v>
@@ -57859,16 +57975,16 @@
         <v>0.167</v>
       </c>
       <c r="D5" t="s" s="46">
-        <v>2074</v>
+        <v>2076</v>
       </c>
       <c r="E5" s="47">
         <f>_xlfn.COUNTIFS('Unit'!$J$3:$J$599,"Yes",'Unit'!$G$3:$G$599,3)+_xlfn.COUNTIFS('Trap'!$J$3:$J$544,"Yes",'Trap'!$G$3:$G$544,3)+_xlfn.COUNTIFS('Tech'!$J$3:$J$545,"Yes",'Tech'!$G$3:$G$545,3)</f>
-        <v>99</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" ht="30.35" customHeight="1">
       <c r="A6" t="s" s="43">
-        <v>2076</v>
+        <v>2078</v>
       </c>
       <c r="B6" s="44">
         <v>16</v>
@@ -57877,16 +57993,16 @@
         <v>0.1</v>
       </c>
       <c r="D6" t="s" s="46">
-        <v>2077</v>
+        <v>2079</v>
       </c>
       <c r="E6" s="47">
         <f>_xlfn.COUNTIFS('Unit'!$J$3:$J$599,"Yes",'Unit'!$G$3:$G$599,4)+_xlfn.COUNTIFS('Trap'!$J$3:$J$544,"Yes",'Trap'!$G$3:$G$544,4)+_xlfn.COUNTIFS('Tech'!$J$3:$J$545,"Yes",'Tech'!$G$3:$G$545,4)</f>
-        <v>57</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" ht="16.35" customHeight="1">
       <c r="A7" t="s" s="48">
-        <v>2078</v>
+        <v>2080</v>
       </c>
       <c r="B7" s="49">
         <v>9</v>
@@ -57895,11 +58011,11 @@
         <v>0.053</v>
       </c>
       <c r="D7" t="s" s="46">
-        <v>2079</v>
+        <v>2081</v>
       </c>
       <c r="E7" s="47">
         <f>_xlfn.COUNTIFS('Unit'!$J$3:$J$599,"Yes",'Unit'!$G$3:$G$599,5)+_xlfn.COUNTIFS('Trap'!$J$3:$J$544,"Yes",'Trap'!$G$3:$G$544,5)+_xlfn.COUNTIFS('Tech'!$J$3:$J$545,"Yes",'Tech'!$G$3:$G$545,5)</f>
-        <v>43</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" ht="16.35" customHeight="1">
@@ -57928,17 +58044,17 @@
         <v>22</v>
       </c>
       <c r="B11" t="s" s="56">
-        <v>2067</v>
+        <v>2069</v>
       </c>
       <c r="C11" s="57"/>
       <c r="D11" s="57"/>
       <c r="E11" t="s" s="58">
-        <v>2070</v>
+        <v>2072</v>
       </c>
     </row>
     <row r="12" ht="16.35" customHeight="1">
       <c r="A12" t="s" s="43">
-        <v>2080</v>
+        <v>2082</v>
       </c>
       <c r="B12" s="44">
         <v>60</v>
@@ -57952,7 +58068,7 @@
     </row>
     <row r="13" ht="16.35" customHeight="1">
       <c r="A13" t="s" s="43">
-        <v>2081</v>
+        <v>2083</v>
       </c>
       <c r="B13" s="44">
         <v>60</v>
@@ -57966,7 +58082,7 @@
     </row>
     <row r="14" ht="16.35" customHeight="1">
       <c r="A14" t="s" s="43">
-        <v>2082</v>
+        <v>2084</v>
       </c>
       <c r="B14" s="44">
         <v>60</v>
@@ -58014,10 +58130,10 @@
     <row r="2" ht="20.25" customHeight="1">
       <c r="A2" s="6"/>
       <c r="B2" t="s" s="5">
-        <v>2083</v>
+        <v>2085</v>
       </c>
       <c r="C2" t="s" s="5">
-        <v>2084</v>
+        <v>2086</v>
       </c>
       <c r="D2" s="6"/>
       <c r="E2" s="6"/>
@@ -58027,10 +58143,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s" s="8">
-        <v>2085</v>
+        <v>2087</v>
       </c>
       <c r="C3" t="s" s="17">
-        <v>2086</v>
+        <v>2088</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -58040,10 +58156,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s" s="11">
-        <v>2087</v>
+        <v>2089</v>
       </c>
       <c r="C4" t="s" s="19">
-        <v>2088</v>
+        <v>2090</v>
       </c>
       <c r="D4" s="12"/>
       <c r="E4" s="12"/>
@@ -58053,10 +58169,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s" s="11">
-        <v>2089</v>
+        <v>2091</v>
       </c>
       <c r="C5" t="s" s="19">
-        <v>2090</v>
+        <v>2092</v>
       </c>
       <c r="D5" s="12"/>
       <c r="E5" s="12"/>
@@ -58066,10 +58182,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s" s="11">
-        <v>2091</v>
+        <v>2093</v>
       </c>
       <c r="C6" t="s" s="19">
-        <v>2091</v>
+        <v>2093</v>
       </c>
       <c r="D6" s="12"/>
       <c r="E6" s="12"/>
@@ -58079,10 +58195,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s" s="11">
-        <v>2092</v>
+        <v>2094</v>
       </c>
       <c r="C7" t="s" s="19">
-        <v>2093</v>
+        <v>2095</v>
       </c>
       <c r="D7" s="12"/>
       <c r="E7" s="12"/>
@@ -58092,10 +58208,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s" s="11">
-        <v>2094</v>
+        <v>2096</v>
       </c>
       <c r="C8" t="s" s="19">
-        <v>2095</v>
+        <v>2097</v>
       </c>
       <c r="D8" s="12"/>
       <c r="E8" s="12"/>
@@ -58105,10 +58221,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="s" s="11">
-        <v>2096</v>
+        <v>2098</v>
       </c>
       <c r="C9" t="s" s="19">
-        <v>2097</v>
+        <v>2099</v>
       </c>
       <c r="D9" s="12"/>
       <c r="E9" s="12"/>
@@ -58118,10 +58234,10 @@
         <v>8</v>
       </c>
       <c r="B10" t="s" s="11">
-        <v>2098</v>
+        <v>2100</v>
       </c>
       <c r="C10" t="s" s="19">
-        <v>2099</v>
+        <v>2101</v>
       </c>
       <c r="D10" s="12"/>
       <c r="E10" s="12"/>

</xml_diff>

<commit_message>
Fix battle prompt races, intercept swaps, Union Maniac, and turn-banner lock.
Await on-expose/reveal chains, physically swap Bat Swarm intercepts, restore Union Maniac after new_game, and block human/AI input until the turn banner dismisses plus 0.2s.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/context/card_data.xlsx
+++ b/context/card_data.xlsx
@@ -31560,10 +31560,10 @@
       </c>
       <c r="C27" s="29"/>
       <c r="D27" s="30">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E27" s="30">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F27" t="s" s="31">
         <v>3</v>

</xml_diff>

<commit_message>
Ship booster rarity weights, Union Cage surround, omen polish, and local content.
Normalize pack weights to rarity, swap four starter-overlapping booster cards, mark their demo flags, and generalize surround-trap triggers for Union Cage. Also includes omen rune/setup UX, card/omen art, exploration/puzzle updates, and related battle wiring.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/context/card_data.xlsx
+++ b/context/card_data.xlsx
@@ -5299,7 +5299,7 @@
     <t>Hostage</t>
   </si>
   <si>
-    <t>You reveal 1 own cell. Until this turn ends, attacker cannot target that cell.</t>
+    <t>Usable when foe attacks. You can reveal one of your unit. Until this turn ends, foe cannot target that unit. If already targeted it, foe must choose other cell.</t>
   </si>
   <si>
     <t>Bait</t>
@@ -5378,7 +5378,7 @@
     <t>Bunker</t>
   </si>
   <si>
-    <t>Attacker cannot target surrounding cells until the end of this turn.</t>
+    <t>Usable when foe attack this card or surround cells. Foe cannot target surrounding cells until the end of this turn. If already targeted, they must choose other cell.</t>
   </si>
   <si>
     <t>Foul Gas</t>
@@ -5618,7 +5618,7 @@
     <t>Self-destruct</t>
   </si>
   <si>
-    <t>You select 1 of your unit. +10 ATK until your turn ends, but also destroy it. You pay no cost.</t>
+    <t>You select 1 of your unit. +50 ATK&amp;DEF until your turn ends, but also destroy it. You pay no cost.</t>
   </si>
   <si>
     <t>Rank C Bounty</t>
@@ -5972,7 +5972,7 @@
     <t>Illustration</t>
   </si>
   <si>
-    <t>Booster Pack - Blightsilver / 3</t>
+    <t>Booster Pack - Blightsilver / 4</t>
   </si>
   <si>
     <t>Booster Pack - Unseen Presence / 2</t>
@@ -10050,7 +10050,9 @@
         <f>(D36*6)+(E36*4)</f>
         <v>1280</v>
       </c>
-      <c r="L36" s="12"/>
+      <c r="L36" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="M36" s="12"/>
       <c r="N36" s="12"/>
       <c r="O36" s="12"/>
@@ -10798,7 +10800,9 @@
         <f>(D54*6)+(E54*4)</f>
         <v>300</v>
       </c>
-      <c r="L54" s="12"/>
+      <c r="L54" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="M54" s="12"/>
       <c r="N54" s="12"/>
       <c r="O54" s="12"/>
@@ -10880,7 +10884,9 @@
         <f>(D56*6)+(E56*4)</f>
         <v>1310</v>
       </c>
-      <c r="L56" s="12"/>
+      <c r="L56" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="M56" s="12"/>
       <c r="N56" s="12"/>
       <c r="O56" s="12"/>
@@ -16553,7 +16559,9 @@
         <f>(D197*6)+(E197*4)</f>
         <v>810</v>
       </c>
-      <c r="L197" s="12"/>
+      <c r="L197" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="M197" s="12"/>
       <c r="N197" s="12"/>
       <c r="O197" s="12"/>
@@ -17863,7 +17871,9 @@
         <f>(D229*6)+(E229*4)</f>
         <v>410</v>
       </c>
-      <c r="L229" s="12"/>
+      <c r="L229" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="M229" s="12"/>
       <c r="N229" s="12"/>
       <c r="O229" s="12"/>
@@ -23462,7 +23472,9 @@
         <v>684</v>
       </c>
       <c r="I369" s="12"/>
-      <c r="J369" s="12"/>
+      <c r="J369" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K369" s="18">
         <f>(D369*6)+(E369*4)</f>
         <v>150</v>
@@ -23499,7 +23511,9 @@
         <v>686</v>
       </c>
       <c r="I370" s="12"/>
-      <c r="J370" s="12"/>
+      <c r="J370" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K370" s="18">
         <f>(D370*6)+(E370*4)</f>
         <v>280</v>
@@ -23536,7 +23550,9 @@
         <v>688</v>
       </c>
       <c r="I371" s="12"/>
-      <c r="J371" s="12"/>
+      <c r="J371" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K371" s="18">
         <f>(D371*6)+(E371*4)</f>
         <v>330</v>
@@ -23616,7 +23632,9 @@
         <v>691</v>
       </c>
       <c r="I373" s="12"/>
-      <c r="J373" s="12"/>
+      <c r="J373" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K373" s="18">
         <f>(D373*6)+(E373*4)</f>
         <v>240</v>
@@ -23653,7 +23671,9 @@
         <v>693</v>
       </c>
       <c r="I374" s="12"/>
-      <c r="J374" s="12"/>
+      <c r="J374" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K374" s="18">
         <f>(D374*6)+(E374*4)</f>
         <v>130</v>
@@ -23776,7 +23796,9 @@
         <v>699</v>
       </c>
       <c r="I377" s="12"/>
-      <c r="J377" s="12"/>
+      <c r="J377" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K377" s="18">
         <f>(D377*6)+(E377*4)</f>
         <v>390</v>
@@ -23813,7 +23835,9 @@
         <v>701</v>
       </c>
       <c r="I378" s="12"/>
-      <c r="J378" s="12"/>
+      <c r="J378" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K378" s="18">
         <f>(D378*6)+(E378*4)</f>
         <v>590</v>
@@ -23850,7 +23874,9 @@
         <v>703</v>
       </c>
       <c r="I379" s="12"/>
-      <c r="J379" s="12"/>
+      <c r="J379" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K379" s="18">
         <f>(D379*6)+(E379*4)</f>
         <v>240</v>
@@ -23887,7 +23913,9 @@
         <v>705</v>
       </c>
       <c r="I380" s="12"/>
-      <c r="J380" s="12"/>
+      <c r="J380" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K380" s="18">
         <f>(D380*6)+(E380*4)</f>
         <v>490</v>
@@ -23924,7 +23952,9 @@
         <v>707</v>
       </c>
       <c r="I381" s="12"/>
-      <c r="J381" s="12"/>
+      <c r="J381" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K381" s="18">
         <f>(D381*6)+(E381*4)</f>
         <v>500</v>
@@ -23961,7 +23991,9 @@
         <v>709</v>
       </c>
       <c r="I382" s="12"/>
-      <c r="J382" s="12"/>
+      <c r="J382" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K382" s="18">
         <f>(D382*6)+(E382*4)</f>
         <v>470</v>
@@ -23998,7 +24030,9 @@
         <v>711</v>
       </c>
       <c r="I383" s="12"/>
-      <c r="J383" s="12"/>
+      <c r="J383" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K383" s="18">
         <f>(D383*6)+(E383*4)</f>
         <v>200</v>
@@ -24082,7 +24116,9 @@
         <v>715</v>
       </c>
       <c r="I385" s="12"/>
-      <c r="J385" s="12"/>
+      <c r="J385" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K385" s="18">
         <f>(D385*6)+(E385*4)</f>
         <v>630</v>
@@ -24119,7 +24155,9 @@
         <v>646</v>
       </c>
       <c r="I386" s="12"/>
-      <c r="J386" s="12"/>
+      <c r="J386" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K386" s="18">
         <f>(D386*6)+(E386*4)</f>
         <v>1300</v>
@@ -24199,7 +24237,9 @@
         <v>720</v>
       </c>
       <c r="I388" s="12"/>
-      <c r="J388" s="12"/>
+      <c r="J388" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K388" s="18">
         <f>(D388*6)+(E388*4)</f>
         <v>790</v>
@@ -24236,7 +24276,9 @@
         <v>722</v>
       </c>
       <c r="I389" s="12"/>
-      <c r="J389" s="12"/>
+      <c r="J389" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K389" s="18">
         <f>(D389*6)+(E389*4)</f>
         <v>0</v>
@@ -24273,7 +24315,9 @@
         <v>724</v>
       </c>
       <c r="I390" s="12"/>
-      <c r="J390" s="12"/>
+      <c r="J390" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K390" s="18">
         <f>(D390*6)+(E390*4)</f>
         <v>600</v>
@@ -24353,7 +24397,9 @@
         <v>39</v>
       </c>
       <c r="I392" s="12"/>
-      <c r="J392" s="12"/>
+      <c r="J392" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K392" s="18">
         <f>(D392*6)+(E392*4)</f>
         <v>1040</v>
@@ -24390,7 +24436,9 @@
         <v>39</v>
       </c>
       <c r="I393" s="12"/>
-      <c r="J393" s="12"/>
+      <c r="J393" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K393" s="18">
         <f>(D393*6)+(E393*4)</f>
         <v>420</v>
@@ -24427,7 +24475,9 @@
         <v>730</v>
       </c>
       <c r="I394" s="12"/>
-      <c r="J394" s="12"/>
+      <c r="J394" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K394" s="18">
         <f>(D394*6)+(E394*4)</f>
         <v>790</v>
@@ -24464,7 +24514,9 @@
         <v>732</v>
       </c>
       <c r="I395" s="12"/>
-      <c r="J395" s="12"/>
+      <c r="J395" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K395" s="18">
         <f>(D395*6)+(E395*4)</f>
         <v>1800</v>
@@ -24501,7 +24553,9 @@
         <v>734</v>
       </c>
       <c r="I396" s="12"/>
-      <c r="J396" s="12"/>
+      <c r="J396" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="K396" s="18">
         <f>(D396*6)+(E396*4)</f>
         <v>980</v>
@@ -35692,7 +35746,7 @@
         <v>1576</v>
       </c>
       <c r="C4" s="18">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="D4" s="12"/>
       <c r="E4" s="12"/>
@@ -36130,7 +36184,7 @@
         <v>1576</v>
       </c>
       <c r="C17" s="18">
-        <v>400</v>
+        <v>800</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="12"/>
@@ -36214,7 +36268,9 @@
         <v>35</v>
       </c>
       <c r="K19" s="12"/>
-      <c r="L19" s="12"/>
+      <c r="L19" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="M19" s="12"/>
       <c r="N19" s="12"/>
       <c r="O19" s="12"/>
@@ -36244,7 +36300,9 @@
         <v>35</v>
       </c>
       <c r="K20" s="12"/>
-      <c r="L20" s="12"/>
+      <c r="L20" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="M20" s="12"/>
       <c r="N20" s="12"/>
       <c r="O20" s="12"/>
@@ -36308,7 +36366,9 @@
         <v>35</v>
       </c>
       <c r="K22" s="12"/>
-      <c r="L22" s="12"/>
+      <c r="L22" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="M22" s="12"/>
       <c r="N22" s="12"/>
       <c r="O22" s="12"/>
@@ -36368,7 +36428,9 @@
         <v>35</v>
       </c>
       <c r="K24" s="12"/>
-      <c r="L24" s="12"/>
+      <c r="L24" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="M24" s="12"/>
       <c r="N24" s="12"/>
       <c r="O24" s="12"/>
@@ -36398,7 +36460,9 @@
         <v>35</v>
       </c>
       <c r="K25" s="12"/>
-      <c r="L25" s="12"/>
+      <c r="L25" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="M25" s="12"/>
       <c r="N25" s="12"/>
       <c r="O25" s="12"/>
@@ -36908,7 +36972,9 @@
         <v>35</v>
       </c>
       <c r="K42" s="12"/>
-      <c r="L42" s="12"/>
+      <c r="L42" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="M42" s="12"/>
       <c r="N42" s="12"/>
       <c r="O42" s="12"/>
@@ -46661,7 +46727,7 @@
   <dimension ref="A1:P545"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="16.3516" style="35" customWidth="1"/>
+    <col min="1" max="1" width="27.7422" style="35" customWidth="1"/>
     <col min="2" max="2" width="9.67188" style="35" customWidth="1"/>
     <col min="3" max="3" width="5.17188" style="35" customWidth="1"/>
     <col min="4" max="4" width="6.17188" style="35" customWidth="1"/>
@@ -47147,7 +47213,9 @@
         <v>35</v>
       </c>
       <c r="K15" s="12"/>
-      <c r="L15" s="12"/>
+      <c r="L15" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="M15" s="12"/>
       <c r="N15" s="12"/>
       <c r="O15" s="12"/>
@@ -47247,7 +47315,9 @@
       <c r="K18" s="12"/>
       <c r="L18" s="12"/>
       <c r="M18" s="12"/>
-      <c r="N18" s="12"/>
+      <c r="N18" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="O18" s="12"/>
       <c r="P18" s="12"/>
     </row>
@@ -47275,7 +47345,9 @@
         <v>35</v>
       </c>
       <c r="K19" s="12"/>
-      <c r="L19" s="12"/>
+      <c r="L19" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="M19" s="12"/>
       <c r="N19" s="12"/>
       <c r="O19" s="12"/>
@@ -47335,7 +47407,9 @@
         <v>35</v>
       </c>
       <c r="K21" s="12"/>
-      <c r="L21" s="12"/>
+      <c r="L21" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="M21" s="12"/>
       <c r="N21" s="12"/>
       <c r="O21" s="12"/>
@@ -47493,7 +47567,9 @@
         <v>35</v>
       </c>
       <c r="K26" s="12"/>
-      <c r="L26" s="12"/>
+      <c r="L26" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="M26" s="12"/>
       <c r="N26" s="12"/>
       <c r="O26" s="12"/>
@@ -57961,7 +58037,7 @@
       </c>
       <c r="E4" s="47">
         <f>_xlfn.COUNTIFS('Unit'!$J$3:$J$599,"Yes",'Unit'!$G$3:$G$599,2)+_xlfn.COUNTIFS('Trap'!$J$3:$J$544,"Yes",'Trap'!$G$3:$G$544,2)+_xlfn.COUNTIFS('Tech'!$J$3:$J$545,"Yes",'Tech'!$G$3:$G$545,2)</f>
-        <v>112</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" ht="16.35" customHeight="1">
@@ -57979,7 +58055,7 @@
       </c>
       <c r="E5" s="47">
         <f>_xlfn.COUNTIFS('Unit'!$J$3:$J$599,"Yes",'Unit'!$G$3:$G$599,3)+_xlfn.COUNTIFS('Trap'!$J$3:$J$544,"Yes",'Trap'!$G$3:$G$544,3)+_xlfn.COUNTIFS('Tech'!$J$3:$J$545,"Yes",'Tech'!$G$3:$G$545,3)</f>
-        <v>104</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" ht="30.35" customHeight="1">
@@ -57997,7 +58073,7 @@
       </c>
       <c r="E6" s="47">
         <f>_xlfn.COUNTIFS('Unit'!$J$3:$J$599,"Yes",'Unit'!$G$3:$G$599,4)+_xlfn.COUNTIFS('Trap'!$J$3:$J$544,"Yes",'Trap'!$G$3:$G$544,4)+_xlfn.COUNTIFS('Tech'!$J$3:$J$545,"Yes",'Tech'!$G$3:$G$545,4)</f>
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" ht="16.35" customHeight="1">
@@ -58015,7 +58091,7 @@
       </c>
       <c r="E7" s="47">
         <f>_xlfn.COUNTIFS('Unit'!$J$3:$J$599,"Yes",'Unit'!$G$3:$G$599,5)+_xlfn.COUNTIFS('Trap'!$J$3:$J$544,"Yes",'Trap'!$G$3:$G$544,5)+_xlfn.COUNTIFS('Tech'!$J$3:$J$545,"Yes",'Tech'!$G$3:$G$545,5)</f>
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" ht="16.35" customHeight="1">
@@ -58063,7 +58139,7 @@
       <c r="D12" s="54"/>
       <c r="E12" s="47">
         <f>_xlfn.COUNTIFS('Unit'!$N$3:$N$599,"Yes")+_xlfn.COUNTIFS('Trap'!$N$3:$N$544,"Yes")+_xlfn.COUNTIFS('Tech'!$N$3:$N$545,"Yes")</f>
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" ht="16.35" customHeight="1">

</xml_diff>

<commit_message>
checkpoint before checking out main
</commit_message>
<xml_diff>
--- a/context/card_data.xlsx
+++ b/context/card_data.xlsx
@@ -5522,7 +5522,7 @@
     <t>Union Cage</t>
   </si>
   <si>
-    <t>If attacker Is Union card, that unit cannot attack until the attacker’s next turn ends.</t>
+    <t>Usable if a Union card attack this card or the surround cell. That Union card cannot attack until the attacker’s next turn ends.</t>
   </si>
   <si>
     <t>Plunder</t>
@@ -8845,7 +8845,9 @@
         <f>(D7*6)+(E7*4)</f>
         <v>780</v>
       </c>
-      <c r="L7" s="12"/>
+      <c r="L7" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="M7" s="12"/>
       <c r="N7" s="12"/>
       <c r="O7" s="12"/>
@@ -11081,7 +11083,9 @@
         <f>(D61*6)+(E61*4)</f>
         <v>830</v>
       </c>
-      <c r="L61" s="12"/>
+      <c r="L61" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="M61" s="12"/>
       <c r="N61" s="12"/>
       <c r="O61" s="12"/>
@@ -36034,7 +36038,9 @@
         <v>35</v>
       </c>
       <c r="K12" s="12"/>
-      <c r="L12" s="12"/>
+      <c r="L12" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="M12" s="12"/>
       <c r="N12" s="12"/>
       <c r="O12" s="12"/>
@@ -36942,7 +36948,9 @@
         <v>35</v>
       </c>
       <c r="K41" s="12"/>
-      <c r="L41" s="12"/>
+      <c r="L41" t="s" s="19">
+        <v>35</v>
+      </c>
       <c r="M41" s="12"/>
       <c r="N41" s="12"/>
       <c r="O41" s="12"/>
@@ -47345,9 +47353,7 @@
         <v>35</v>
       </c>
       <c r="K19" s="12"/>
-      <c r="L19" t="s" s="19">
-        <v>35</v>
-      </c>
+      <c r="L19" s="12"/>
       <c r="M19" s="12"/>
       <c r="N19" s="12"/>
       <c r="O19" s="12"/>
@@ -47487,7 +47493,7 @@
         <v>1806</v>
       </c>
       <c r="C24" s="18">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D24" s="12"/>
       <c r="E24" s="12"/>
@@ -47551,7 +47557,7 @@
         <v>1806</v>
       </c>
       <c r="C26" s="18">
-        <v>2000</v>
+        <v>900</v>
       </c>
       <c r="D26" s="12"/>
       <c r="E26" s="12"/>
@@ -48585,7 +48591,7 @@
         <v>1806</v>
       </c>
       <c r="C62" s="18">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D62" s="12"/>
       <c r="E62" s="12"/>

</xml_diff>